<commit_message>
first sibling iz eksela dodata f-ja
</commit_message>
<xml_diff>
--- a/testdata/data.xlsx
+++ b/testdata/data.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="8400"/>
+    <workbookView windowWidth="22188" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="67">
   <si>
     <t>username</t>
   </si>
@@ -77,7 +77,7 @@
     <t>saving_account_bban</t>
   </si>
   <si>
-    <t>saving_account_2_bban</t>
+    <t>racunZaUplatu</t>
   </si>
   <si>
     <t>search_purpose</t>
@@ -92,24 +92,27 @@
     <t>credit_card_number</t>
   </si>
   <si>
-    <t>credit_card_2_name</t>
-  </si>
-  <si>
-    <t>credit_card_2_number</t>
-  </si>
-  <si>
-    <t>loan_account_bban</t>
-  </si>
-  <si>
-    <t>loan_account_name</t>
-  </si>
-  <si>
-    <t>term_deposit_bban</t>
-  </si>
-  <si>
     <t>term_deposit_name</t>
   </si>
   <si>
+    <t>Broj_identifikacionog_dokumenta</t>
+  </si>
+  <si>
+    <t>Datum_važenja_identifikacionog_dokumenta</t>
+  </si>
+  <si>
+    <t>Adresa_iz_identifikacionog_dokumenta</t>
+  </si>
+  <si>
+    <t>Kucni_telefon</t>
+  </si>
+  <si>
+    <t>Mobilni_telefon</t>
+  </si>
+  <si>
+    <t>E-mail_adresa</t>
+  </si>
+  <si>
     <t>Osir ANOEV</t>
   </si>
   <si>
@@ -155,7 +158,7 @@
     <t>9011008384007</t>
   </si>
   <si>
-    <t>9011008395360</t>
+    <t>105059203100439109</t>
   </si>
   <si>
     <t>Naknada za TR</t>
@@ -170,13 +173,22 @@
     <t>4431********0118</t>
   </si>
   <si>
-    <t>Visa revolving card</t>
-  </si>
-  <si>
-    <t>4176********8476</t>
-  </si>
-  <si>
-    <t>205-9032022325800-66</t>
+    <t>012879003</t>
+  </si>
+  <si>
+    <t>09.08.2033</t>
+  </si>
+  <si>
+    <t>ŽILA VERNA 10/1-12</t>
+  </si>
+  <si>
+    <t>00112522735</t>
+  </si>
+  <si>
+    <t>+381612468647</t>
+  </si>
+  <si>
+    <t>zadruga.racunovodja@gmail.com</t>
   </si>
   <si>
     <t>Enil ČIĆVI</t>
@@ -216,12 +228,6 @@
   </si>
   <si>
     <t>Jail ĆEVGIMILĆ</t>
-  </si>
-  <si>
-    <t>205-0049032401456-48</t>
-  </si>
-  <si>
-    <t>Gotovinski kredit</t>
   </si>
 </sst>
 </file>
@@ -273,13 +279,21 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="11"/>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FF800080"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -291,14 +305,6 @@
       <color rgb="FF800080"/>
       <name val="Calibri"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -750,12 +756,12 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
@@ -880,11 +886,14 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
@@ -902,25 +911,34 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" quotePrefix="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" quotePrefix="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1" quotePrefix="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1" quotePrefix="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1242,7 +1260,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AA6"/>
+  <dimension ref="A1:AB6"/>
   <sheetFormatPr defaultColWidth="8.87962962962963" defaultRowHeight="14.4" outlineLevelRow="5"/>
   <cols>
     <col min="1" max="1" width="17.75" customWidth="1"/>
@@ -1259,23 +1277,27 @@
     <col min="13" max="15" width="30.4259259259259" style="1" customWidth="1"/>
     <col min="16" max="16" width="19.8888888888889" style="1" customWidth="1"/>
     <col min="17" max="19" width="24.6666666666667" style="1" customWidth="1"/>
-    <col min="20" max="24" width="33.2222222222222" style="1" customWidth="1"/>
-    <col min="25" max="25" width="31.1111111111111" style="1" customWidth="1"/>
-    <col min="26" max="26" width="33.2222222222222" style="1" customWidth="1"/>
-    <col min="27" max="27" width="19.1111111111111" style="1" customWidth="1"/>
+    <col min="20" max="21" width="33.2222222222222" style="1" customWidth="1"/>
+    <col min="22" max="22" width="19.1111111111111" style="1" customWidth="1"/>
+    <col min="23" max="23" width="29.7777777777778" customWidth="1"/>
+    <col min="24" max="24" width="40.1111111111111" customWidth="1"/>
+    <col min="25" max="25" width="34.7777777777778" customWidth="1"/>
+    <col min="26" max="26" width="13.2222222222222" customWidth="1"/>
+    <col min="27" max="27" width="15.2222222222222" style="2" customWidth="1"/>
+    <col min="28" max="28" width="31.2222222222222" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="1" spans="1:27">
-      <c r="A1" s="2" t="s">
+    <row r="1" customFormat="1" spans="1:28">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -1314,16 +1336,16 @@
       <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="Q1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="R1" s="4" t="s">
         <v>17</v>
       </c>
       <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="T1" s="4" t="s">
         <v>19</v>
       </c>
       <c r="U1" s="1" t="s">
@@ -1332,370 +1354,338 @@
       <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" s="2" t="s">
         <v>26</v>
       </c>
+      <c r="AB1" t="s">
+        <v>27</v>
+      </c>
     </row>
-    <row r="2" customFormat="1" spans="1:27">
-      <c r="A2" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B2" s="4" t="s">
+    <row r="2" customFormat="1" spans="1:28">
+      <c r="A2" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="B2" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="E2" s="11" t="s">
+      <c r="D2" s="3" t="s">
         <v>31</v>
       </c>
+      <c r="E2" s="14" t="s">
+        <v>32</v>
+      </c>
       <c r="F2" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="P2" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q2" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="R2" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="S2" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="T2" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="V2" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="H2" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="P2" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q2" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="R2" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="S2" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="T2" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="U2" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="V2" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="W2" s="1" t="s">
+      <c r="W2" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="X2" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y2" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="Z2" s="6" t="s">
+      <c r="X2" t="s">
         <v>49</v>
       </c>
-      <c r="AA2" s="6" t="s">
-        <v>32</v>
+      <c r="Y2" t="s">
+        <v>50</v>
+      </c>
+      <c r="Z2" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="AA2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="AB2" s="8" t="s">
+        <v>53</v>
       </c>
     </row>
-    <row r="3" customFormat="1" spans="1:27">
+    <row r="3" customFormat="1" spans="1:28">
       <c r="A3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C3" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="E3" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>52</v>
+      <c r="D3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E3" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>56</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="I3" s="11" t="s">
-        <v>54</v>
+        <v>57</v>
+      </c>
+      <c r="I3" s="14" t="s">
+        <v>58</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q3" s="1"/>
       <c r="R3" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="S3" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="T3" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="U3" s="1"/>
-      <c r="V3" s="1"/>
-      <c r="W3" s="1"/>
-      <c r="X3" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y3" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="Z3" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="AA3" s="1" t="s">
-        <v>35</v>
-      </c>
+      <c r="V3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA3" s="2"/>
     </row>
-    <row r="4" customFormat="1" spans="1:27">
+    <row r="4" customFormat="1" spans="1:28">
       <c r="A4" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C4" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="E4" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>35</v>
+      <c r="D4" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>36</v>
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="K4" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="N4" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="L4" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="N4" s="1" t="s">
-        <v>55</v>
-      </c>
       <c r="O4" s="1" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q4" s="1"/>
       <c r="R4" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="S4" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="T4" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="U4" s="1"/>
-      <c r="V4" s="1"/>
-      <c r="W4" s="1"/>
-      <c r="X4" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y4" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="Z4" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="AA4" s="1" t="s">
-        <v>35</v>
-      </c>
+      <c r="V4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA4" s="2"/>
     </row>
-    <row r="5" customFormat="1" spans="1:27">
+    <row r="5" customFormat="1" spans="1:28">
       <c r="A5" t="s">
-        <v>61</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="F5" s="9" t="s">
-        <v>35</v>
+      <c r="D5" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>36</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q5" s="1"/>
       <c r="R5" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="S5" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="T5" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="U5" s="1"/>
-      <c r="V5" s="1"/>
-      <c r="W5" s="1"/>
-      <c r="X5" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y5" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="Z5" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="AA5" s="1" t="s">
-        <v>35</v>
-      </c>
+      <c r="V5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA5" s="2"/>
     </row>
-    <row r="6" s="1" customFormat="1" spans="1:27">
+    <row r="6" s="1" customFormat="1" spans="1:28">
       <c r="A6" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>28</v>
+        <v>66</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>29</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="R6" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="S6" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="T6" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="X6" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="Y6" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="Z6" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="AA6" s="1" t="s">
-        <v>35</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="V6" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA6" s="13"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1704,6 +1694,7 @@
     <hyperlink ref="B4" r:id="rId1" display="https://uat.dbp.nlb.si/web-retail/login" tooltip="https://uat.dbp.nlb.si/web-retail/login"/>
     <hyperlink ref="B5" r:id="rId1" display="https://uat.dbp.nlb.si/web-retail/login" tooltip="https://uat.dbp.nlb.si/web-retail/login"/>
     <hyperlink ref="B6" r:id="rId1" display="https://uat.dbp.nlb.si/web-retail/login" tooltip="https://uat.dbp.nlb.si/web-retail/login"/>
+    <hyperlink ref="AB2" r:id="rId2" display="zadruga.racunovodja@gmail.com"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
data dodavanje podataka za ljiljanu kovac
</commit_message>
<xml_diff>
--- a/testdata/data.xlsx
+++ b/testdata/data.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9588"/>
+    <workbookView windowWidth="13140" windowHeight="6732"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,11 +27,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="29">
   <si>
     <t>username</t>
   </si>
   <si>
+    <t>password</t>
+  </si>
+  <si>
     <t>webpage</t>
   </si>
   <si>
@@ -47,67 +50,25 @@
     <t>cardNumber</t>
   </si>
   <si>
-    <t>term_deposit_account_details_opening_date</t>
-  </si>
-  <si>
-    <t>term_deposit_account_details_expiration_date</t>
-  </si>
-  <si>
-    <t>maturity_account</t>
-  </si>
-  <si>
-    <t>currentDomesticAccountName</t>
-  </si>
-  <si>
-    <t>currentDomesticAccountBBAN</t>
-  </si>
-  <si>
-    <t>personal_account_bban</t>
-  </si>
-  <si>
-    <t>personal_account_name</t>
-  </si>
-  <si>
-    <t>second_personal_account_name</t>
-  </si>
-  <si>
-    <t>second_personal_account_bban</t>
-  </si>
-  <si>
-    <t>saving_account_bban</t>
-  </si>
-  <si>
-    <t>saving_account_2_bban</t>
-  </si>
-  <si>
-    <t>search_purpose</t>
-  </si>
-  <si>
-    <t>saving_account_name</t>
-  </si>
-  <si>
-    <t>credit_card_name</t>
-  </si>
-  <si>
-    <t>credit_card_number</t>
-  </si>
-  <si>
-    <t>credit_card_2_name</t>
-  </si>
-  <si>
-    <t>credit_card_2_number</t>
-  </si>
-  <si>
-    <t>loan_account_bban</t>
-  </si>
-  <si>
-    <t>loan_account_name</t>
-  </si>
-  <si>
-    <t>term_deposit_bban</t>
-  </si>
-  <si>
-    <t>term_deposit_name</t>
+    <t>Tip_identifikacionog_dokumenta</t>
+  </si>
+  <si>
+    <t>Broj_identifikacionog_dokumenta</t>
+  </si>
+  <si>
+    <t>Datum_važenja_identifikacionog_dokumenta</t>
+  </si>
+  <si>
+    <t>Adresa_iz_identifikacionog_dokumenta</t>
+  </si>
+  <si>
+    <t>Kucni_telefon</t>
+  </si>
+  <si>
+    <t>Mobilni_telefon</t>
+  </si>
+  <si>
+    <t>E-mail_adresa</t>
   </si>
   <si>
     <t>snezana.nikolic</t>
@@ -128,61 +89,31 @@
     <t>989122******5440</t>
   </si>
   <si>
-    <t>15. 1. 2016</t>
-  </si>
-  <si>
-    <t>15. 1. 2028</t>
+    <t>ljiljanakovac</t>
   </si>
   <si>
     <t>.</t>
   </si>
   <si>
-    <t>205-9001007790944-88</t>
-  </si>
-  <si>
-    <t>RS35 2059 0310 0441 9532 81</t>
-  </si>
-  <si>
-    <t>Foreign currency payment accounts</t>
-  </si>
-  <si>
-    <t>Devizni platni račun</t>
-  </si>
-  <si>
-    <t>RS35 2059 0310 0441 7882 84</t>
-  </si>
-  <si>
-    <t>9011008384007</t>
-  </si>
-  <si>
-    <t>9011008395360</t>
-  </si>
-  <si>
-    <t>Naknada za TR</t>
-  </si>
-  <si>
-    <t>A vista depozitni račun</t>
-  </si>
-  <si>
-    <t>Visa prepaid</t>
-  </si>
-  <si>
-    <t>4431********0118</t>
-  </si>
-  <si>
-    <t>Visa revolving card</t>
-  </si>
-  <si>
-    <t>4176********8476</t>
-  </si>
-  <si>
-    <t>205-9032022325800-66</t>
-  </si>
-  <si>
-    <t>Oročeni depozit</t>
-  </si>
-  <si>
-    <t>ljiljanakovac</t>
+    <t>Lična karta</t>
+  </si>
+  <si>
+    <t>012879003</t>
+  </si>
+  <si>
+    <t>09.08.2033</t>
+  </si>
+  <si>
+    <t>ŽILA VERNA 10/1-12</t>
+  </si>
+  <si>
+    <t>00112522735</t>
+  </si>
+  <si>
+    <t>+381612468647</t>
+  </si>
+  <si>
+    <t>zadruga.racunovodja@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -195,7 +126,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -211,11 +142,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
@@ -228,15 +154,9 @@
       <charset val="0"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="10"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color theme="1"/>
-      <name val="Segoe UI"/>
+      <name val="Courier New"/>
       <charset val="134"/>
     </font>
     <font>
@@ -704,133 +624,133 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -838,12 +758,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
@@ -853,13 +773,13 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" quotePrefix="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1181,7 +1101,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AB3"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr defaultColWidth="8.87962962962963" defaultRowHeight="14.4" outlineLevelRow="2"/>
   <cols>
     <col min="1" max="1" width="17.75" customWidth="1"/>
@@ -1190,217 +1110,131 @@
     <col min="5" max="5" width="11.25" customWidth="1"/>
     <col min="6" max="6" width="22.4444444444444" customWidth="1"/>
     <col min="7" max="7" width="17.5555555555556" customWidth="1"/>
-    <col min="8" max="8" width="42.1111111111111" customWidth="1"/>
-    <col min="9" max="9" width="44.1111111111111" customWidth="1"/>
-    <col min="10" max="11" width="33.8888888888889" customWidth="1"/>
-    <col min="12" max="12" width="28.8888888888889" customWidth="1"/>
-    <col min="13" max="13" width="27.8888888888889" style="1" customWidth="1"/>
-    <col min="14" max="16" width="30.4259259259259" style="1" customWidth="1"/>
-    <col min="17" max="17" width="19.8888888888889" style="1" customWidth="1"/>
-    <col min="18" max="20" width="24.6666666666667" style="1" customWidth="1"/>
-    <col min="21" max="25" width="33.2222222222222" style="1" customWidth="1"/>
-    <col min="26" max="26" width="31.1111111111111" style="1" customWidth="1"/>
-    <col min="27" max="27" width="33.2222222222222" style="1" customWidth="1"/>
-    <col min="28" max="28" width="19.1111111111111" style="1" customWidth="1"/>
+    <col min="8" max="8" width="30.6666666666667" customWidth="1"/>
+    <col min="9" max="9" width="31.6666666666667" customWidth="1"/>
+    <col min="10" max="10" width="42" customWidth="1"/>
+    <col min="11" max="11" width="36.6666666666667" customWidth="1"/>
+    <col min="12" max="12" width="13.2222222222222" customWidth="1"/>
+    <col min="13" max="13" width="15.2222222222222" customWidth="1"/>
+    <col min="14" max="14" width="31.2222222222222" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="1" spans="1:28">
-      <c r="A1" s="2" t="s">
+    <row r="1" customFormat="1" spans="1:14">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="1" t="s">
+    </row>
+    <row r="2" customFormat="1" spans="1:14">
+      <c r="A2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="B2" s="3">
+        <v>9128</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="D2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="E2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="F2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="V1" s="1" t="s">
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" t="s">
         <v>20</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="B3" s="3">
+        <v>2804</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" t="s">
         <v>21</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="G3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="I3" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="J3" t="s">
         <v>24</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="K3" t="s">
         <v>25</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="L3" s="8" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="2" customFormat="1" spans="1:28">
-      <c r="A2" s="2" t="s">
+      <c r="M3" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="4">
-        <v>9128</v>
-      </c>
-      <c r="C2" s="5" t="s">
+      <c r="N3" s="7" t="s">
         <v>28</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="L2" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q2" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="R2" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="S2" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="T2" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="U2" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="V2" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="W2" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="X2" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y2" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="Z2" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="AA2" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="AB2" s="7" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="3" spans="1:28">
-      <c r="A3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B3" s="4">
-        <v>2804</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="F3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G3" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" display="https://uat.dbp.nlb.si/web-retail/login" tooltip="https://uat.dbp.nlb.si/web-retail/login"/>
     <hyperlink ref="C3" r:id="rId1" display="https://uat.dbp.nlb.si/web-retail/login" tooltip="https://uat.dbp.nlb.si/web-retail/login"/>
+    <hyperlink ref="N3" r:id="rId2" display="zadruga.racunovodja@gmail.com"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
change name of account - done
</commit_message>
<xml_diff>
--- a/testdata/data.xlsx
+++ b/testdata/data.xlsx
@@ -168,7 +168,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -208,12 +208,6 @@
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color theme="1"/>
-      <name val="Segoe UI"/>
-      <charset val="134"/>
     </font>
     <font>
       <u/>
@@ -675,134 +669,134 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -828,9 +822,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="6" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1">
@@ -1155,8 +1146,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:U6"/>
-  <sheetFormatPr defaultColWidth="8.87962962962963" defaultRowHeight="14.4" outlineLevelRow="5"/>
+  <dimension ref="A1:U3"/>
+  <sheetFormatPr defaultColWidth="8.87962962962963" defaultRowHeight="14.4" outlineLevelRow="2"/>
   <cols>
     <col min="1" max="1" width="17.75" customWidth="1"/>
     <col min="2" max="3" width="35.5555555555556" customWidth="1"/>
@@ -1175,6 +1166,7 @@
     <col min="18" max="18" width="16.2222222222222" customWidth="1"/>
     <col min="19" max="19" width="22.4444444444444" customWidth="1"/>
     <col min="20" max="20" width="22.7777777777778" customWidth="1"/>
+    <col min="21" max="21" width="33.1111111111111" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="1" spans="1:21">
@@ -1335,7 +1327,7 @@
       <c r="I3" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="J3" s="10" t="s">
+      <c r="J3" s="9" t="s">
         <v>36</v>
       </c>
       <c r="K3" t="s">
@@ -1344,7 +1336,7 @@
       <c r="L3" t="s">
         <v>38</v>
       </c>
-      <c r="M3" s="10" t="s">
+      <c r="M3" s="9" t="s">
         <v>39</v>
       </c>
       <c r="N3" s="5" t="s">
@@ -1371,9 +1363,6 @@
       <c r="U3" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="6" spans="1:21">
-      <c r="Q6" s="9"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
transakcije i quick actions pocetno
</commit_message>
<xml_diff>
--- a/testdata/data.xlsx
+++ b/testdata/data.xlsx
@@ -77,13 +77,13 @@
     <t>nazivRacunaRSD</t>
   </si>
   <si>
-    <t>racunRSD</t>
+    <t>brojRacunaRSD</t>
   </si>
   <si>
     <t>nazivRacunaRSD2</t>
   </si>
   <si>
-    <t>racunRSD2</t>
+    <t>brojRacunaRSD2</t>
   </si>
   <si>
     <t>nazivRacunaEUR</t>

</xml_diff>